<commit_message>
fix: resolve duplicate IDs and add conversion settings
- Fix answer code and field name collisions
- Add ConversionConfig options for welcome/end
  notes, other pattern, and markdown
- Refactor converter with row builder and
  language loop helpers
- Document configuration options in README
</commit_message>
<xml_diff>
--- a/docker_tests/fixtures/all_types_survey.xlsx
+++ b/docker_tests/fixtures/all_types_survey.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -717,18 +717,42 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>end_group</v>
+        <v>select_one yesno</v>
+      </c>
+      <c r="B29" t="str">
+        <v>q_minimal</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v>Bevorzugst du Dropdown?</v>
+      </c>
+      <c r="E29" t="str">
+        <v>minimal</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>begin_group</v>
-      </c>
-      <c r="B30" t="str">
-        <v>matrix_wrapper</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Selbsteinschätzung technischer Fähigkeiten</v>
+        <v>end_group</v>
       </c>
     </row>
     <row r="31">
@@ -736,27 +760,24 @@
         <v>begin_group</v>
       </c>
       <c r="B31" t="str">
-        <v>matrix_inner</v>
+        <v>matrix_wrapper</v>
       </c>
       <c r="D31" t="str">
-        <v>Programmierkenntnisse</v>
-      </c>
-      <c r="E31" t="str">
-        <v>field-list</v>
+        <v>Selbsteinschätzung technischer Fähigkeiten</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>select_one proficiency</v>
+        <v>begin_group</v>
       </c>
       <c r="B32" t="str">
-        <v>matrix_header</v>
+        <v>matrix_inner</v>
       </c>
       <c r="D32" t="str">
-        <v>Wie schätzen Sie Ihre Kenntnisse ein?</v>
+        <v>Programmierkenntnisse</v>
       </c>
       <c r="E32" t="str">
-        <v>label</v>
+        <v>field-list</v>
       </c>
     </row>
     <row r="33">
@@ -764,13 +785,13 @@
         <v>select_one proficiency</v>
       </c>
       <c r="B33" t="str">
-        <v>skill_python</v>
+        <v>matrix_header</v>
       </c>
       <c r="D33" t="str">
-        <v>Python</v>
+        <v>Wie schätzen Sie Ihre Kenntnisse ein?</v>
       </c>
       <c r="E33" t="str">
-        <v>list-nolabel</v>
+        <v>label</v>
       </c>
     </row>
     <row r="34">
@@ -778,10 +799,10 @@
         <v>select_one proficiency</v>
       </c>
       <c r="B34" t="str">
-        <v>skill_js</v>
+        <v>skill_python</v>
       </c>
       <c r="D34" t="str">
-        <v>JavaScript</v>
+        <v>Python</v>
       </c>
       <c r="E34" t="str">
         <v>list-nolabel</v>
@@ -792,10 +813,10 @@
         <v>select_one proficiency</v>
       </c>
       <c r="B35" t="str">
-        <v>skill_sql</v>
+        <v>skill_js</v>
       </c>
       <c r="D35" t="str">
-        <v>SQL</v>
+        <v>JavaScript</v>
       </c>
       <c r="E35" t="str">
         <v>list-nolabel</v>
@@ -803,7 +824,16 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>end_group</v>
+        <v>select_one proficiency</v>
+      </c>
+      <c r="B36" t="str">
+        <v>skill_sql</v>
+      </c>
+      <c r="D36" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="E36" t="str">
+        <v>list-nolabel</v>
       </c>
     </row>
     <row r="37">
@@ -813,76 +843,67 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>begin_group</v>
-      </c>
-      <c r="B38" t="str">
-        <v>or_other_types</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Weitere Fragen</v>
+        <v>end_group</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>select_one topics or_other</v>
+        <v>begin_group</v>
       </c>
       <c r="B39" t="str">
-        <v>q_sel1_other</v>
+        <v>or_other_types</v>
       </c>
       <c r="D39" t="str">
-        <v>Welcher Track hat Ihnen am besten gefallen?</v>
+        <v>Weitere Fragen</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>select_multiple topics or_other</v>
+        <v>select_one topics or_other</v>
       </c>
       <c r="B40" t="str">
-        <v>q_selm_other</v>
+        <v>q_sel1_other</v>
       </c>
       <c r="D40" t="str">
-        <v>Welche Tracks würden Sie erneut besuchen?</v>
+        <v>Welcher Track hat Ihnen am besten gefallen?</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>rank aspects or_other</v>
+        <v>select_multiple topics or_other</v>
       </c>
       <c r="B41" t="str">
-        <v>q_rank_other</v>
+        <v>q_selm_other</v>
       </c>
       <c r="D41" t="str">
-        <v>Was hat Ihnen an der Veranstaltung am meisten gebracht?</v>
+        <v>Welche Tracks würden Sie erneut besuchen?</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>end_group</v>
+        <v>rank aspects or_other</v>
+      </c>
+      <c r="B42" t="str">
+        <v>q_rank_other</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Was hat Ihnen an der Veranstaltung am meisten gebracht?</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>begin_group</v>
-      </c>
-      <c r="B43" t="str">
-        <v>features</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Anmeldedaten</v>
+        <v>end_group</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>text</v>
+        <v>begin_group</v>
       </c>
       <c r="B44" t="str">
-        <v>q_mandatory</v>
+        <v>features</v>
       </c>
       <c r="D44" t="str">
-        <v>Wie lautet Ihre E-Mail-Adresse?</v>
-      </c>
-      <c r="F44" t="str">
-        <v>yes</v>
+        <v>Anmeldedaten</v>
       </c>
     </row>
     <row r="45">
@@ -890,44 +911,44 @@
         <v>text</v>
       </c>
       <c r="B45" t="str">
-        <v>q_hint</v>
+        <v>q_mandatory</v>
       </c>
       <c r="D45" t="str">
-        <v>Wie lautet Ihre Telefonnummer?</v>
-      </c>
-      <c r="G45" t="str">
-        <v>Format: +49 123 456789</v>
+        <v>Wie lautet Ihre E-Mail-Adresse?</v>
+      </c>
+      <c r="F45" t="str">
+        <v>yes</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>integer</v>
+        <v>text</v>
       </c>
       <c r="B46" t="str">
-        <v>q_constraint</v>
+        <v>q_hint</v>
       </c>
       <c r="D46" t="str">
-        <v>Wie alt sind Sie?</v>
-      </c>
-      <c r="H46" t="str">
-        <v>. &gt;= 18 and . &lt;= 120</v>
-      </c>
-      <c r="I46" t="str">
-        <v>Bitte geben Sie ein gültiges Alter zwischen 18 und 120 ein</v>
+        <v>Wie lautet Ihre Telefonnummer?</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Format: +49 123 456789</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>text</v>
+        <v>integer</v>
       </c>
       <c r="B47" t="str">
-        <v>q_default</v>
+        <v>q_constraint</v>
       </c>
       <c r="D47" t="str">
-        <v>In welchem Land leben Sie?</v>
-      </c>
-      <c r="J47" t="str">
-        <v>Deutschland</v>
+        <v>Wie alt sind Sie?</v>
+      </c>
+      <c r="H47" t="str">
+        <v>. &gt;= 18 and . &lt;= 120</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Bitte geben Sie ein gültiges Alter zwischen 18 und 120 ein</v>
       </c>
     </row>
     <row r="48">
@@ -935,13 +956,13 @@
         <v>text</v>
       </c>
       <c r="B48" t="str">
-        <v>q_relevant</v>
+        <v>q_default</v>
       </c>
       <c r="D48" t="str">
-        <v>Wie sollen wir Sie kontaktieren?</v>
-      </c>
-      <c r="K48" t="str">
-        <v>${q_mandatory} != ''</v>
+        <v>In welchem Land leben Sie?</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Deutschland</v>
       </c>
     </row>
     <row r="49">
@@ -949,19 +970,10 @@
         <v>text</v>
       </c>
       <c r="B49" t="str">
-        <v>q_all_features</v>
+        <v>q_relevant</v>
       </c>
       <c r="D49" t="str">
-        <v>Haben Sie noch Anmerkungen?</v>
-      </c>
-      <c r="F49" t="str">
-        <v>yes</v>
-      </c>
-      <c r="G49" t="str">
-        <v>Freiwillig, aber willkommen</v>
-      </c>
-      <c r="J49" t="str">
-        <v>Keine Anmerkungen</v>
+        <v>Wie sollen wir Sie kontaktieren?</v>
       </c>
       <c r="K49" t="str">
         <v>${q_mandatory} != ''</v>
@@ -969,23 +981,46 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>end_group</v>
+        <v>text</v>
+      </c>
+      <c r="B50" t="str">
+        <v>q_all_features</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Haben Sie noch Anmerkungen?</v>
+      </c>
+      <c r="F50" t="str">
+        <v>yes</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Freiwillig, aber willkommen</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Keine Anmerkungen</v>
+      </c>
+      <c r="K50" t="str">
+        <v>${q_mandatory} != ''</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
+        <v>end_group</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
         <v>note</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B52" t="str">
         <v>orphan_after</v>
       </c>
-      <c r="D51" t="str">
+      <c r="D52" t="str">
         <v>Vielen Dank für Ihre Teilnahme an dieser Umfrage!</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>